<commit_message>
fix(data): normalize APR financial values to RSD
</commit_message>
<xml_diff>
--- a/docs/Market Intelligence/01_Market_Data/APR/Processed/apr_data_quality_1039_4631_2026-07-22.xlsx
+++ b/docs/Market Intelligence/01_Market_Data/APR/Processed/apr_data_quality_1039_4631_2026-07-22.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,6 +550,16 @@
         <v>0</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>financial_multiplier_applied</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>